<commit_message>
Verify canonical Windows paths and make helper coverage visible in the sample
</commit_message>
<xml_diff>
--- a/samples/sample_requests_2026-11.xlsx
+++ b/samples/sample_requests_2026-11.xlsx
@@ -2455,9 +2455,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">休</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
@@ -2769,9 +2769,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">休</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">

</xml_diff>